<commit_message>
Update ExT settlement report and inventory features
</commit_message>
<xml_diff>
--- a/ExT 재고매입.xlsx
+++ b/ExT 재고매입.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\NGS결산\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{375E567A-252C-4667-8EC6-17BB477FD56F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6647620-1105-4D03-97E8-8788210FF08A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
   <si>
     <t>구매전표</t>
   </si>
@@ -233,6 +233,18 @@
     </r>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+      </rPr>
+      <t>합계</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -241,7 +253,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="#,##0_ "/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -308,6 +320,12 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -317,7 +335,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -383,13 +401,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -450,10 +505,28 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -770,36 +843,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="10.59765625" customWidth="1" collapsed="1"/>
     <col min="2" max="2" width="50" customWidth="1" collapsed="1"/>
     <col min="3" max="3" width="7.8984375" customWidth="1" collapsed="1"/>
     <col min="4" max="6" width="14.8984375" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="13.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="12" t="s">
         <v>18</v>
       </c>
@@ -808,7 +882,7 @@
         <v>618832500</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -824,11 +898,14 @@
       <c r="E6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="22" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G6" s="26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -844,11 +921,15 @@
       <c r="E7" s="6">
         <v>85000000</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="23">
         <v>8500000</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G7" s="27">
+        <f>E7+F7</f>
+        <v>93500000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -864,11 +945,15 @@
       <c r="E8" s="6">
         <v>21675000</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="23">
         <v>2167500</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G8" s="27">
+        <f t="shared" ref="G8:G19" si="0">E8+F8</f>
+        <v>23842500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
@@ -884,11 +969,15 @@
       <c r="E9" s="6">
         <v>4200000</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="23">
         <v>420000</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G9" s="27">
+        <f t="shared" si="0"/>
+        <v>4620000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
@@ -904,11 +993,15 @@
       <c r="E10" s="6">
         <v>0</v>
       </c>
-      <c r="F10" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="F10" s="23">
+        <v>0</v>
+      </c>
+      <c r="G10" s="27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -924,11 +1017,15 @@
       <c r="E11" s="6">
         <v>4200000</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="23">
         <v>420000</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G11" s="27">
+        <f t="shared" si="0"/>
+        <v>4620000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
@@ -944,11 +1041,15 @@
       <c r="E12" s="6">
         <v>0</v>
       </c>
-      <c r="F12" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="F12" s="23">
+        <v>0</v>
+      </c>
+      <c r="G12" s="27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
@@ -964,11 +1065,15 @@
       <c r="E13" s="6">
         <v>25000000</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="23">
         <v>2500000</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G13" s="27">
+        <f t="shared" si="0"/>
+        <v>27500000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="3" t="s">
         <v>9</v>
       </c>
@@ -984,11 +1089,15 @@
       <c r="E14" s="6">
         <v>0</v>
       </c>
-      <c r="F14" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="F14" s="23">
+        <v>0</v>
+      </c>
+      <c r="G14" s="27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>9</v>
       </c>
@@ -1004,11 +1113,15 @@
       <c r="E15" s="6">
         <v>25000000</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="23">
         <v>2500000</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G15" s="27">
+        <f t="shared" si="0"/>
+        <v>27500000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>9</v>
       </c>
@@ -1024,11 +1137,15 @@
       <c r="E16" s="6">
         <v>0</v>
       </c>
-      <c r="F16" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="F16" s="23">
+        <v>0</v>
+      </c>
+      <c r="G16" s="27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A17" s="8" t="s">
         <v>9</v>
       </c>
@@ -1044,11 +1161,15 @@
       <c r="E17" s="11">
         <v>85000000</v>
       </c>
-      <c r="F17" s="11">
+      <c r="F17" s="23">
         <v>8500000</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G17" s="27">
+        <f t="shared" si="0"/>
+        <v>93500000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A18" s="8" t="s">
         <v>9</v>
       </c>
@@ -1064,11 +1185,15 @@
       <c r="E18" s="11">
         <v>175000000</v>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="23">
         <v>17500000</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G18" s="27">
+        <f t="shared" si="0"/>
+        <v>192500000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A19" s="15" t="s">
         <v>9</v>
       </c>
@@ -1084,11 +1209,15 @@
       <c r="E19" s="18">
         <v>137500000</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="24">
         <v>13750000</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="G19" s="27">
+        <f t="shared" si="0"/>
+        <v>151250000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A20" s="19"/>
       <c r="B20" s="20" t="s">
         <v>19</v>
@@ -1098,19 +1227,23 @@
         <v>339</v>
       </c>
       <c r="D20" s="21">
-        <f t="shared" ref="D20:F20" si="0">SUM(D7:D19)</f>
+        <f t="shared" ref="D20:G20" si="1">SUM(D7:D19)</f>
         <v>30065000</v>
       </c>
       <c r="E20" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>562575000</v>
       </c>
-      <c r="F20" s="21">
-        <f t="shared" si="0"/>
+      <c r="F20" s="25">
+        <f t="shared" si="1"/>
         <v>56257500</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.4"/>
+      <c r="G20" s="25">
+        <f t="shared" si="1"/>
+        <v>618832500</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>